<commit_message>
Added labels for manual delivery in and out.
</commit_message>
<xml_diff>
--- a/Files/Controls.xlsx
+++ b/Files/Controls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\NVDA\VismaAdministration\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D8B9246-DD08-4391-A200-437D5C9D8CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA87390-790B-4A54-9E61-0C4ED34C4F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1425" yWindow="1425" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1919" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1985" uniqueCount="545">
   <si>
     <t>WindowClassName</t>
   </si>
@@ -1653,6 +1653,21 @@
   </si>
   <si>
     <t>Lösenord</t>
+  </si>
+  <si>
+    <t>Lönummer</t>
+  </si>
+  <si>
+    <t>Antal</t>
+  </si>
+  <si>
+    <t>Pris styck</t>
+  </si>
+  <si>
+    <t>Frakt styck</t>
+  </si>
+  <si>
+    <t>Kommentar</t>
   </si>
 </sst>
 </file>
@@ -1971,7 +1986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E710"/>
+  <dimension ref="A1:E732"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
@@ -11282,6 +11297,314 @@
         <v>539</v>
       </c>
     </row>
+    <row r="711" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A711" t="s">
+        <v>6</v>
+      </c>
+      <c r="B711">
+        <v>22825</v>
+      </c>
+      <c r="C711" t="s">
+        <v>254</v>
+      </c>
+      <c r="D711" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="712" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A712" t="s">
+        <v>6</v>
+      </c>
+      <c r="B712">
+        <v>22818</v>
+      </c>
+      <c r="C712" t="s">
+        <v>254</v>
+      </c>
+      <c r="D712" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="713" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A713" t="s">
+        <v>6</v>
+      </c>
+      <c r="B713">
+        <v>22828</v>
+      </c>
+      <c r="C713" t="s">
+        <v>254</v>
+      </c>
+      <c r="D713" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="714" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A714" t="s">
+        <v>6</v>
+      </c>
+      <c r="B714">
+        <v>22613</v>
+      </c>
+      <c r="C714" t="s">
+        <v>254</v>
+      </c>
+      <c r="D714" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="715" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A715" t="s">
+        <v>6</v>
+      </c>
+      <c r="B715">
+        <v>22619</v>
+      </c>
+      <c r="C715" t="s">
+        <v>254</v>
+      </c>
+      <c r="D715" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="716" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A716" t="s">
+        <v>6</v>
+      </c>
+      <c r="B716">
+        <v>22831</v>
+      </c>
+      <c r="C716" t="s">
+        <v>254</v>
+      </c>
+      <c r="D716" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="717" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A717" t="s">
+        <v>6</v>
+      </c>
+      <c r="B717">
+        <v>22834</v>
+      </c>
+      <c r="C717" t="s">
+        <v>254</v>
+      </c>
+      <c r="D717" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="718" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A718" t="s">
+        <v>6</v>
+      </c>
+      <c r="B718">
+        <v>22835</v>
+      </c>
+      <c r="C718" t="s">
+        <v>254</v>
+      </c>
+      <c r="D718" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="719" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A719" t="s">
+        <v>6</v>
+      </c>
+      <c r="B719">
+        <v>22846</v>
+      </c>
+      <c r="C719" t="s">
+        <v>254</v>
+      </c>
+      <c r="D719" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="720" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A720" t="s">
+        <v>6</v>
+      </c>
+      <c r="B720">
+        <v>22843</v>
+      </c>
+      <c r="C720" t="s">
+        <v>254</v>
+      </c>
+      <c r="D720" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="721" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A721" t="s">
+        <v>6</v>
+      </c>
+      <c r="B721">
+        <v>22844</v>
+      </c>
+      <c r="C721" t="s">
+        <v>254</v>
+      </c>
+      <c r="D721" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="722" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A722" t="s">
+        <v>6</v>
+      </c>
+      <c r="B722">
+        <v>22845</v>
+      </c>
+      <c r="C722" t="s">
+        <v>254</v>
+      </c>
+      <c r="D722" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="723" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A723" t="s">
+        <v>6</v>
+      </c>
+      <c r="B723">
+        <v>22825</v>
+      </c>
+      <c r="C723" t="s">
+        <v>256</v>
+      </c>
+      <c r="D723" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="724" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A724" t="s">
+        <v>6</v>
+      </c>
+      <c r="B724">
+        <v>22818</v>
+      </c>
+      <c r="C724" t="s">
+        <v>256</v>
+      </c>
+      <c r="D724" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="725" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A725" t="s">
+        <v>6</v>
+      </c>
+      <c r="B725">
+        <v>22828</v>
+      </c>
+      <c r="C725" t="s">
+        <v>256</v>
+      </c>
+      <c r="D725" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="726" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A726" t="s">
+        <v>6</v>
+      </c>
+      <c r="B726">
+        <v>22613</v>
+      </c>
+      <c r="C726" t="s">
+        <v>256</v>
+      </c>
+      <c r="D726" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="727" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A727" t="s">
+        <v>6</v>
+      </c>
+      <c r="B727">
+        <v>22619</v>
+      </c>
+      <c r="C727" t="s">
+        <v>256</v>
+      </c>
+      <c r="D727" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="728" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A728" t="s">
+        <v>6</v>
+      </c>
+      <c r="B728">
+        <v>22831</v>
+      </c>
+      <c r="C728" t="s">
+        <v>256</v>
+      </c>
+      <c r="D728" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="729" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A729" t="s">
+        <v>6</v>
+      </c>
+      <c r="B729">
+        <v>22846</v>
+      </c>
+      <c r="C729" t="s">
+        <v>256</v>
+      </c>
+      <c r="D729" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="730" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A730" t="s">
+        <v>6</v>
+      </c>
+      <c r="B730">
+        <v>22843</v>
+      </c>
+      <c r="C730" t="s">
+        <v>256</v>
+      </c>
+      <c r="D730" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="731" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A731" t="s">
+        <v>6</v>
+      </c>
+      <c r="B731">
+        <v>22844</v>
+      </c>
+      <c r="C731" t="s">
+        <v>256</v>
+      </c>
+      <c r="D731" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="732" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A732" t="s">
+        <v>6</v>
+      </c>
+      <c r="B732">
+        <v>22845</v>
+      </c>
+      <c r="C732" t="s">
+        <v>256</v>
+      </c>
+      <c r="D732" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added more control labels.
</commit_message>
<xml_diff>
--- a/Files/Controls.xlsx
+++ b/Files/Controls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\NVDA\VismaAdministration\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA87390-790B-4A54-9E61-0C4ED34C4F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C259FE-284F-4572-92A6-76F4C897C2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="1425" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1985" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1997" uniqueCount="546">
   <si>
     <t>WindowClassName</t>
   </si>
@@ -1668,6 +1668,9 @@
   </si>
   <si>
     <t>Kommentar</t>
+  </si>
+  <si>
+    <t>Anmärkning 3</t>
   </si>
 </sst>
 </file>
@@ -1986,7 +1989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E732"/>
+  <dimension ref="A1:E736"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
@@ -11605,6 +11608,62 @@
         <v>63</v>
       </c>
     </row>
+    <row r="733" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A733" t="s">
+        <v>6</v>
+      </c>
+      <c r="B733">
+        <v>24583</v>
+      </c>
+      <c r="C733" t="s">
+        <v>250</v>
+      </c>
+      <c r="D733" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="734" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A734" t="s">
+        <v>6</v>
+      </c>
+      <c r="B734">
+        <v>23261</v>
+      </c>
+      <c r="C734" t="s">
+        <v>250</v>
+      </c>
+      <c r="D734" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="735" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A735" t="s">
+        <v>6</v>
+      </c>
+      <c r="B735">
+        <v>23262</v>
+      </c>
+      <c r="C735" t="s">
+        <v>250</v>
+      </c>
+      <c r="D735" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="736" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A736" t="s">
+        <v>6</v>
+      </c>
+      <c r="B736">
+        <v>23263</v>
+      </c>
+      <c r="C736" t="s">
+        <v>250</v>
+      </c>
+      <c r="D736" t="s">
+        <v>545</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new control labels and fixed some that was broken.
</commit_message>
<xml_diff>
--- a/Files/Controls.xlsx
+++ b/Files/Controls.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\NVDA\VismaAdministration\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C259FE-284F-4572-92A6-76F4C897C2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77FBB7D1-1CAD-4A33-8F3E-DA955BEEA3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1997" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2030" uniqueCount="546">
   <si>
     <t>WindowClassName</t>
   </si>
@@ -2456,6 +2456,9 @@
       <c r="B34">
         <v>22613</v>
       </c>
+      <c r="C34" t="s">
+        <v>243</v>
+      </c>
       <c r="D34" t="s">
         <v>8</v>
       </c>
@@ -2467,6 +2470,9 @@
       <c r="B35">
         <v>22614</v>
       </c>
+      <c r="C35" t="s">
+        <v>243</v>
+      </c>
       <c r="D35" t="s">
         <v>9</v>
       </c>
@@ -2478,6 +2484,9 @@
       <c r="B36">
         <v>22615</v>
       </c>
+      <c r="C36" t="s">
+        <v>243</v>
+      </c>
       <c r="D36" t="s">
         <v>10</v>
       </c>
@@ -2489,6 +2498,9 @@
       <c r="B37">
         <v>22616</v>
       </c>
+      <c r="C37" t="s">
+        <v>243</v>
+      </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
@@ -2500,6 +2512,9 @@
       <c r="B38">
         <v>22619</v>
       </c>
+      <c r="C38" t="s">
+        <v>243</v>
+      </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
@@ -2511,6 +2526,9 @@
       <c r="B39">
         <v>22617</v>
       </c>
+      <c r="C39" t="s">
+        <v>243</v>
+      </c>
       <c r="D39" t="s">
         <v>13</v>
       </c>
@@ -2521,6 +2539,9 @@
       </c>
       <c r="B40">
         <v>22709</v>
+      </c>
+      <c r="C40" t="s">
+        <v>243</v>
       </c>
       <c r="D40" t="s">
         <v>14</v>
@@ -2533,6 +2554,9 @@
       <c r="B41">
         <v>21657</v>
       </c>
+      <c r="C41" t="s">
+        <v>243</v>
+      </c>
       <c r="D41" t="s">
         <v>16</v>
       </c>
@@ -2544,6 +2568,9 @@
       <c r="B42">
         <v>22620</v>
       </c>
+      <c r="C42" t="s">
+        <v>243</v>
+      </c>
       <c r="D42" t="s">
         <v>17</v>
       </c>
@@ -2554,6 +2581,9 @@
       </c>
       <c r="B43">
         <v>22643</v>
+      </c>
+      <c r="C43" t="s">
+        <v>243</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
@@ -2566,6 +2596,9 @@
       <c r="B44">
         <v>22641</v>
       </c>
+      <c r="C44" t="s">
+        <v>243</v>
+      </c>
       <c r="D44" t="s">
         <v>20</v>
       </c>
@@ -2577,6 +2610,9 @@
       <c r="B45">
         <v>22618</v>
       </c>
+      <c r="C45" t="s">
+        <v>243</v>
+      </c>
       <c r="D45" t="s">
         <v>21</v>
       </c>
@@ -2588,6 +2624,9 @@
       <c r="B46">
         <v>22652</v>
       </c>
+      <c r="C46" t="s">
+        <v>243</v>
+      </c>
       <c r="D46" t="s">
         <v>22</v>
       </c>
@@ -2599,6 +2638,9 @@
       <c r="B47">
         <v>25050</v>
       </c>
+      <c r="C47" t="s">
+        <v>243</v>
+      </c>
       <c r="D47" t="s">
         <v>23</v>
       </c>
@@ -2610,6 +2652,9 @@
       <c r="B48">
         <v>23606</v>
       </c>
+      <c r="C48" t="s">
+        <v>243</v>
+      </c>
       <c r="D48" t="s">
         <v>24</v>
       </c>
@@ -2621,6 +2666,9 @@
       <c r="B49">
         <v>22708</v>
       </c>
+      <c r="C49" t="s">
+        <v>243</v>
+      </c>
       <c r="D49" t="s">
         <v>25</v>
       </c>
@@ -2632,6 +2680,9 @@
       <c r="B50">
         <v>22644</v>
       </c>
+      <c r="C50" t="s">
+        <v>243</v>
+      </c>
       <c r="D50" t="s">
         <v>26</v>
       </c>
@@ -2643,6 +2694,9 @@
       <c r="B51">
         <v>22645</v>
       </c>
+      <c r="C51" t="s">
+        <v>243</v>
+      </c>
       <c r="D51" t="s">
         <v>27</v>
       </c>
@@ -2654,6 +2708,9 @@
       <c r="B52">
         <v>20593</v>
       </c>
+      <c r="C52" t="s">
+        <v>243</v>
+      </c>
       <c r="D52" t="s">
         <v>296</v>
       </c>
@@ -2665,6 +2722,9 @@
       <c r="B53">
         <v>24279</v>
       </c>
+      <c r="C53" t="s">
+        <v>243</v>
+      </c>
       <c r="D53" t="s">
         <v>33</v>
       </c>
@@ -2679,6 +2739,9 @@
       <c r="B54">
         <v>22642</v>
       </c>
+      <c r="C54" t="s">
+        <v>243</v>
+      </c>
       <c r="D54" t="s">
         <v>34</v>
       </c>
@@ -2690,6 +2753,9 @@
       <c r="B55">
         <v>22628</v>
       </c>
+      <c r="C55" t="s">
+        <v>243</v>
+      </c>
       <c r="D55" t="s">
         <v>35</v>
       </c>
@@ -2701,6 +2767,9 @@
       <c r="B56">
         <v>22629</v>
       </c>
+      <c r="C56" t="s">
+        <v>243</v>
+      </c>
       <c r="D56" t="s">
         <v>36</v>
       </c>
@@ -2711,6 +2780,9 @@
       </c>
       <c r="B57">
         <v>22630</v>
+      </c>
+      <c r="C57" t="s">
+        <v>243</v>
       </c>
       <c r="D57" t="s">
         <v>37</v>
@@ -2723,6 +2795,9 @@
       <c r="B58">
         <v>22657</v>
       </c>
+      <c r="C58" t="s">
+        <v>243</v>
+      </c>
       <c r="D58" t="s">
         <v>38</v>
       </c>
@@ -2734,6 +2809,9 @@
       <c r="B59">
         <v>22627</v>
       </c>
+      <c r="C59" t="s">
+        <v>243</v>
+      </c>
       <c r="D59" t="s">
         <v>40</v>
       </c>
@@ -2748,6 +2826,9 @@
       <c r="B60">
         <v>22631</v>
       </c>
+      <c r="C60" t="s">
+        <v>243</v>
+      </c>
       <c r="D60" t="s">
         <v>41</v>
       </c>
@@ -2759,6 +2840,9 @@
       <c r="B61">
         <v>22653</v>
       </c>
+      <c r="C61" t="s">
+        <v>243</v>
+      </c>
       <c r="D61" t="s">
         <v>42</v>
       </c>
@@ -2770,6 +2854,9 @@
       <c r="B62">
         <v>22654</v>
       </c>
+      <c r="C62" t="s">
+        <v>243</v>
+      </c>
       <c r="D62" t="s">
         <v>43</v>
       </c>
@@ -2781,6 +2868,9 @@
       <c r="B63">
         <v>22655</v>
       </c>
+      <c r="C63" t="s">
+        <v>243</v>
+      </c>
       <c r="D63" t="s">
         <v>44</v>
       </c>
@@ -2792,6 +2882,9 @@
       <c r="B64">
         <v>22623</v>
       </c>
+      <c r="C64" t="s">
+        <v>243</v>
+      </c>
       <c r="D64" t="s">
         <v>45</v>
       </c>
@@ -2803,6 +2896,9 @@
       <c r="B65">
         <v>22625</v>
       </c>
+      <c r="C65" t="s">
+        <v>243</v>
+      </c>
       <c r="D65" t="s">
         <v>46</v>
       </c>
@@ -2813,6 +2909,9 @@
       </c>
       <c r="B66">
         <v>22624</v>
+      </c>
+      <c r="C66" t="s">
+        <v>243</v>
       </c>
       <c r="D66" t="s">
         <v>47</v>

</xml_diff>